<commit_message>
Add DCF valuation and target-return tabs to office model
DCF tab discounts remaining lease cashflows plus a 2030 reversion (configurable
discount rate and exit cap rate). Target Return tab solves for the sale price
needed to hit a target annual return and tabulates ROI/annualised return per
sale price. DCF cross-checks at ~AED 6.23M, consistent with the cap-rate range.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F34pBmQnkApCzfs23gFMM6
</commit_message>
<xml_diff>
--- a/Dubai_Office_Valuation.xlsx
+++ b/Dubai_Office_Valuation.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Lease Schedule" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Valuation" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Net Proceeds" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DCF Valuation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Target Return" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,12 +21,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;AED&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="+#,##0 &quot;AED&quot;;-#,##0 &quot;AED&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +71,19 @@
     </font>
     <font>
       <color rgb="00A6A6A6"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00548235"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="9">
@@ -138,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -238,6 +255,42 @@
     </xf>
     <xf numFmtId="166" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1288,4 +1341,730 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DCF VALUATION  —  remaining lease cashflows + 2030 reversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>INPUTS (edit gold)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Discount rate</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Investor's required return</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Exit cap rate (2030)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Yield a buyer pays at resale</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Annual service charge</t>
+        </is>
+      </c>
+      <c r="B6" s="9">
+        <f>Assumptions!B7</f>
+        <v/>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>From Assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Lease Year</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Annual Rent</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Net Rent</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Period t</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Disc. Factor</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>PV of Net Rent</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="20">
+        <f>'Lease Schedule'!C5</f>
+        <v/>
+      </c>
+      <c r="C9" s="20">
+        <f>B9-$B$6</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>A9-Assumptions!$B$8+1</f>
+        <v/>
+      </c>
+      <c r="E9" s="38">
+        <f>IF(D9&lt;1,0,1/(1+$B$4)^D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="20">
+        <f>C9*E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="6">
+        <f>'Lease Schedule'!C6</f>
+        <v/>
+      </c>
+      <c r="C10" s="6">
+        <f>B10-$B$6</f>
+        <v/>
+      </c>
+      <c r="D10" s="12">
+        <f>A10-Assumptions!$B$8+1</f>
+        <v/>
+      </c>
+      <c r="E10" s="39">
+        <f>IF(D10&lt;1,0,1/(1+$B$4)^D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="6">
+        <f>C10*E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="20">
+        <f>'Lease Schedule'!C7</f>
+        <v/>
+      </c>
+      <c r="C11" s="20">
+        <f>B11-$B$6</f>
+        <v/>
+      </c>
+      <c r="D11" s="18">
+        <f>A11-Assumptions!$B$8+1</f>
+        <v/>
+      </c>
+      <c r="E11" s="38">
+        <f>IF(D11&lt;1,0,1/(1+$B$4)^D11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="20">
+        <f>C11*E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="6">
+        <f>'Lease Schedule'!C8</f>
+        <v/>
+      </c>
+      <c r="C12" s="6">
+        <f>B12-$B$6</f>
+        <v/>
+      </c>
+      <c r="D12" s="12">
+        <f>A12-Assumptions!$B$8+1</f>
+        <v/>
+      </c>
+      <c r="E12" s="39">
+        <f>IF(D12&lt;1,0,1/(1+$B$4)^D12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="6">
+        <f>C12*E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="20">
+        <f>'Lease Schedule'!C9</f>
+        <v/>
+      </c>
+      <c r="C13" s="20">
+        <f>B13-$B$6</f>
+        <v/>
+      </c>
+      <c r="D13" s="18">
+        <f>A13-Assumptions!$B$8+1</f>
+        <v/>
+      </c>
+      <c r="E13" s="38">
+        <f>IF(D13&lt;1,0,1/(1+$B$4)^D13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="20">
+        <f>C13*E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" s="40" t="inlineStr">
+        <is>
+          <t>PV of lease income</t>
+        </is>
+      </c>
+      <c r="F14" s="24">
+        <f>SUM(F9:F13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>REVERSION (sale at end of lease, May 2030)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Year-5 net rent</t>
+        </is>
+      </c>
+      <c r="B17" s="42">
+        <f>C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Gross reversion value</t>
+        </is>
+      </c>
+      <c r="B18" s="42">
+        <f>B17/$B$5</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f> Year-5 net rent ÷ exit cap rate</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Period at reversion</t>
+        </is>
+      </c>
+      <c r="B19" s="43">
+        <f>5-Assumptions!B8+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>PV of reversion</t>
+        </is>
+      </c>
+      <c r="B20" s="9">
+        <f>B18/(1+$B$4)^B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>DCF VALUE (today)</t>
+        </is>
+      </c>
+      <c r="B22" s="45">
+        <f>F14+B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Implied gain vs purchase</t>
+        </is>
+      </c>
+      <c r="B23" s="46">
+        <f>B22-Assumptions!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>DCF cross-checks the cap-rate method by valuing the actual remaining cashflows plus a 2030 resale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Lower discount rate → higher value. Lower exit cap → higher reversion. Try 8%/7.5% for an optimistic case.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TARGET RETURN  —  what price hits your goal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>INPUTS (edit gold)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Your cost (purchase price)</t>
+        </is>
+      </c>
+      <c r="B4" s="9">
+        <f>Assumptions!B5</f>
+        <v/>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>From Assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Holding period (years)</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>From buy (~May 2025) to sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Net rent collected while holding</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>449292</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>≈ one year net rent; adjust to actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Agent commission +VAT</t>
+        </is>
+      </c>
+      <c r="B7" s="48">
+        <f>Assumptions!B9*(1+Assumptions!B10)</f>
+        <v/>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>2% x 1.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>TARGET annual return</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Your goal (compound, on cost)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="31" t="inlineStr">
+        <is>
+          <t>Required sale price for target</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Required total profit</t>
+        </is>
+      </c>
+      <c r="B11" s="42">
+        <f>B4*((1+B8)^B5-1)</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f> cost × ((1+target)^years − 1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>Required sale price</t>
+        </is>
+      </c>
+      <c r="B12" s="45">
+        <f>(B11+B4-B6)/(1-B7)</f>
+        <v/>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Price needed to achieve the target return above</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>SCENARIO TABLE — return at each sale price</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Sale Price</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Selling Cost</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Capital Gain</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Total Profit</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Simple ROI</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Annualised</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="B16" s="6">
+        <f>A16*B7</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>A16-B4</f>
+        <v/>
+      </c>
+      <c r="D16" s="36">
+        <f>A16-B16-B4+B6</f>
+        <v/>
+      </c>
+      <c r="E16" s="17">
+        <f>D16/B4</f>
+        <v/>
+      </c>
+      <c r="F16" s="50">
+        <f>(1+E16)^(1/B5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>5900000</v>
+      </c>
+      <c r="B17" s="20">
+        <f>A17*B7</f>
+        <v/>
+      </c>
+      <c r="C17" s="20">
+        <f>A17-B4</f>
+        <v/>
+      </c>
+      <c r="D17" s="33">
+        <f>A17-B17-B4+B6</f>
+        <v/>
+      </c>
+      <c r="E17" s="21">
+        <f>D17/B4</f>
+        <v/>
+      </c>
+      <c r="F17" s="51">
+        <f>(1+E17)^(1/B5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="B18" s="6">
+        <f>A18*B7</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>A18-B4</f>
+        <v/>
+      </c>
+      <c r="D18" s="36">
+        <f>A18-B18-B4+B6</f>
+        <v/>
+      </c>
+      <c r="E18" s="17">
+        <f>D18/B4</f>
+        <v/>
+      </c>
+      <c r="F18" s="50">
+        <f>(1+E18)^(1/B5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>6300000</v>
+      </c>
+      <c r="B19" s="20">
+        <f>A19*B7</f>
+        <v/>
+      </c>
+      <c r="C19" s="20">
+        <f>A19-B4</f>
+        <v/>
+      </c>
+      <c r="D19" s="33">
+        <f>A19-B19-B4+B6</f>
+        <v/>
+      </c>
+      <c r="E19" s="21">
+        <f>D19/B4</f>
+        <v/>
+      </c>
+      <c r="F19" s="51">
+        <f>(1+E19)^(1/B5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="B20" s="6">
+        <f>A20*B7</f>
+        <v/>
+      </c>
+      <c r="C20" s="6">
+        <f>A20-B4</f>
+        <v/>
+      </c>
+      <c r="D20" s="36">
+        <f>A20-B20-B4+B6</f>
+        <v/>
+      </c>
+      <c r="E20" s="17">
+        <f>D20/B4</f>
+        <v/>
+      </c>
+      <c r="F20" s="50">
+        <f>(1+E20)^(1/B5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>6700000</v>
+      </c>
+      <c r="B21" s="20">
+        <f>A21*B7</f>
+        <v/>
+      </c>
+      <c r="C21" s="20">
+        <f>A21-B4</f>
+        <v/>
+      </c>
+      <c r="D21" s="33">
+        <f>A21-B21-B4+B6</f>
+        <v/>
+      </c>
+      <c r="E21" s="21">
+        <f>D21/B4</f>
+        <v/>
+      </c>
+      <c r="F21" s="51">
+        <f>(1+E21)^(1/B5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="B22" s="6">
+        <f>A22*B7</f>
+        <v/>
+      </c>
+      <c r="C22" s="6">
+        <f>A22-B4</f>
+        <v/>
+      </c>
+      <c r="D22" s="36">
+        <f>A22-B22-B4+B6</f>
+        <v/>
+      </c>
+      <c r="E22" s="17">
+        <f>D22/B4</f>
+        <v/>
+      </c>
+      <c r="F22" s="50">
+        <f>(1+E22)^(1/B5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Total Profit = capital gain − selling cost + net rent collected. Annualised compounds Simple ROI over the holding period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Note: ignores DLD transfer fee (buyer-paid) and assumes no mortgage.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add printable Summary cover sheet to office model
One-page landscape summary as the first tab: property facts, three valuation
methods (cap-rate net/gross + DCF), recommendation, outcome at settlement, plus
selling-points and next-steps panels. All figures pull live from the other tabs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F34pBmQnkApCzfs23gFMM6
</commit_message>
<xml_diff>
--- a/Dubai_Office_Valuation.xlsx
+++ b/Dubai_Office_Valuation.xlsx
@@ -7,14 +7,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lease Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Valuation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Net Proceeds" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="DCF Valuation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Target Return" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lease Schedule" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Valuation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Net Proceeds" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DCF Valuation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Target Return" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Summary'!$A$1:$D$24</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -28,7 +31,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,6 +87,23 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="9">
@@ -155,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -291,6 +311,34 @@
     </xf>
     <xf numFmtId="165" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -655,6 +703,290 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="52" t="inlineStr">
+        <is>
+          <t>TENANTED OFFICE — VALUATION SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>Lease May 2025–May 2030 · 5% annual escalation · owner-paid service charge · no mortgage</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>THE PROPERTY</t>
+        </is>
+      </c>
+      <c r="D4" s="54" t="inlineStr">
+        <is>
+          <t>WHY IT'S WORTH MORE THAN YOU PAID</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="55" t="inlineStr">
+        <is>
+          <t>Purchase price (your cost)</t>
+        </is>
+      </c>
+      <c r="B5" s="56">
+        <f>Assumptions!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="55" t="inlineStr">
+        <is>
+          <t>Current passing rent (Year 2)</t>
+        </is>
+      </c>
+      <c r="B6" s="56">
+        <f>Assumptions!B11</f>
+        <v/>
+      </c>
+      <c r="D6" s="57" t="inlineStr">
+        <is>
+          <t>• You bought at an 11% yield; market trades at 7–9%, so the same income is worth more.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="55" t="inlineStr">
+        <is>
+          <t>Annual service charge</t>
+        </is>
+      </c>
+      <c r="B7" s="56">
+        <f>Assumptions!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="55" t="inlineStr">
+        <is>
+          <t>Net operating income (NOI)</t>
+        </is>
+      </c>
+      <c r="B8" s="58">
+        <f>Assumptions!B12</f>
+        <v/>
+      </c>
+      <c r="D8" s="57" t="inlineStr">
+        <is>
+          <t>• 5% annual rent escalation = built-in income growth and inflation hedge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="55" t="inlineStr">
+        <is>
+          <t>Net yield on your cost</t>
+        </is>
+      </c>
+      <c r="B9" s="59">
+        <f>Assumptions!B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="D10" s="57" t="inlineStr">
+        <is>
+          <t>• Secured tenant to May 2030 → income security justifies a sharper yield.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>WHAT IT'S WORTH (three methods)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="55" t="inlineStr">
+        <is>
+          <t>Cap rate – net @ 8.0%</t>
+        </is>
+      </c>
+      <c r="B12" s="56">
+        <f>Valuation!C8</f>
+        <v/>
+      </c>
+      <c r="D12" s="57" t="inlineStr">
+        <is>
+          <t>• Service charge only ~8% of rent, so net yield stays strong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="55" t="inlineStr">
+        <is>
+          <t>Cap rate – gross @ 7.5%</t>
+        </is>
+      </c>
+      <c r="B13" s="56">
+        <f>Valuation!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="55" t="inlineStr">
+        <is>
+          <t>DCF (9% discount / 8% exit)</t>
+        </is>
+      </c>
+      <c r="B14" s="58">
+        <f>DCF Valuation!B22</f>
+        <v/>
+      </c>
+      <c r="D14" s="57" t="inlineStr">
+        <is>
+          <t>• No mortgage → clean title, faster transfer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
+          <t>RECOMMENDATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>List at</t>
+        </is>
+      </c>
+      <c r="B17" s="60" t="inlineStr">
+        <is>
+          <t>AED 6.4M – 6.7M</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>NEXT STEPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Expect to settle</t>
+        </is>
+      </c>
+      <c r="B18" s="60" t="inlineStr">
+        <is>
+          <t>AED 5.9M – 6.3M</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" s="57" t="inlineStr">
+        <is>
+          <t>1. Get a RICS valuation to confirm (~AED 3–6k).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>YOUR OUTCOME (settle ≈ AED 6.0M)</t>
+        </is>
+      </c>
+      <c r="D20" s="57" t="inlineStr">
+        <is>
+          <t>2. Time the sale near May to capture the next 5% step-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="55" t="inlineStr">
+        <is>
+          <t>Net to you after 2% comm.+VAT</t>
+        </is>
+      </c>
+      <c r="B21" s="58">
+        <f>Net Proceeds!D7</f>
+        <v/>
+      </c>
+      <c r="D21" s="57" t="inlineStr">
+        <is>
+          <t>3. List on Property Finder / Bayut with a Trakheesi permit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="55" t="inlineStr">
+        <is>
+          <t>Gain vs purchase</t>
+        </is>
+      </c>
+      <c r="B22" s="61">
+        <f>Net Proceeds!E7</f>
+        <v/>
+      </c>
+      <c r="D22" s="57" t="inlineStr">
+        <is>
+          <t>4. Market the secured income + escalation as the headline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>All figures recalculate from the Assumptions tab. DLD 4% transfer fee normally paid by buyer (excluded). Estimates only — not a formal valuation.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D22"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="D20"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="D21"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="D19"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D14:D15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C14"/>
@@ -824,7 +1156,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -982,7 +1314,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1165,7 +1497,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1343,7 +1675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1687,7 +2019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>